<commit_message>
cross linking of databases
</commit_message>
<xml_diff>
--- a/chromadb/docs/dual_qnas.xlsx
+++ b/chromadb/docs/dual_qnas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\PycharmProjects\gatech-practicum\chromadb\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manis\PycharmProjects\gatech-practicum\chromadb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E959ADD-C5A6-41E3-A15D-5CB07D194144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF36ECC-DD7B-46DD-BB67-93643298472F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QnAs" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
   <si>
     <t>Question</t>
   </si>
@@ -142,10 +142,25 @@
     <t>It depends on your schedule and workload. Dual enrollment can give you a more challenging academic schedule, but you can still participate in extracurriculars if you manage your time effectively.</t>
   </si>
   <si>
-    <t>How do I register for dual enrollment courses?</t>
-  </si>
-  <si>
-    <t>After getting approval from your school and the partnering college, you will typically need to complete a registration process through the college, which may include submitting transcripts, placement tests, or other documentation.</t>
+    <t>scholarships</t>
+  </si>
+  <si>
+    <t>We have two major scholarships available - HOPE Scholarship &amp; Zell Miller Scholarship.The HOPE (Helping Outstanding Pupils Educationally) Scholarship is a Georgia state-funded program that provides financial assistance to Georgia residents to attend in-state colleges and universities based on academic achievement.The Zell Miller Scholarship is a more competitive Georgia state-funded scholarship that offers higher financial aid amounts than the HOPE Scholarship and is based on even stricter eligibility requirements. See here for more information - https://www.gafutures.org/hope-state-aid-programs/hope-zell-miller-scholarships/</t>
+  </si>
+  <si>
+    <t>academic standing</t>
+  </si>
+  <si>
+    <t>What's your Student ID ?</t>
+  </si>
+  <si>
+    <t>graduation</t>
+  </si>
+  <si>
+    <t>To graduate, you must complete a certain number of credits in required subjects (e.g., English, math, science, social studies), pass state exams, and fulfill any additional requirements set by your school.</t>
+  </si>
+  <si>
+    <t>graduation requirements</t>
   </si>
 </sst>
 </file>
@@ -986,13 +1001,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B21"/>
-  <sheetFormatPr defaultColWidth="43.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr defaultColWidth="43.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="77.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="77.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1000,7 +1015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1008,7 +1023,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1016,7 +1031,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1024,7 +1039,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1032,7 +1047,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1040,7 +1055,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1048,7 +1063,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -1056,7 +1071,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1064,7 +1079,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -1072,7 +1087,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1080,7 +1095,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1088,7 +1103,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1096,7 +1111,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1104,7 +1119,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -1112,7 +1127,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -1120,7 +1135,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -1128,7 +1143,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -1136,7 +1151,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -1144,7 +1159,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -1152,12 +1167,36 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>40</v>
       </c>
       <c r="B21" t="s">
         <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>